<commit_message>
Tarik ha pagato 100 euro il 04/04/2026, fino ad aprile pagato, resto in basta per eventuali cambiamenti di prezzo
</commit_message>
<xml_diff>
--- a/Netflix.xlsx
+++ b/Netflix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Netflix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8007BA0-1FB3-4E8D-A9F4-142CD0F9E9E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502F7452-39B6-4395-8121-F63A007271F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="9">
   <si>
     <t>MESE</t>
   </si>
@@ -938,7 +938,7 @@
         <v>2</v>
       </c>
       <c r="Z2" s="2">
-        <f t="shared" ref="Z2:BU2" si="3">ROUND(AL8/AL9,  1)</f>
+        <f t="shared" ref="Z2:BT2" si="3">ROUND(AL8/AL9,  1)</f>
         <v>5</v>
       </c>
       <c r="AA2" s="2">
@@ -1290,24 +1290,20 @@
       <c r="AK3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AL3" s="2">
-        <f t="shared" ref="AI3:BM3" si="5">ROUND(AX8/AX9,  1)</f>
-        <v>5</v>
-      </c>
-      <c r="AM3" s="2">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="AN3" s="2">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="AO3" s="2">
-        <f t="shared" si="5"/>
-        <v>5</v>
+      <c r="AL3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AM3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AN3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AO3" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="AP3" s="2">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="AL3:BM3" si="5">ROUND(BB8/BB9,  1)</f>
         <v>5</v>
       </c>
       <c r="AQ3" s="2">
@@ -1403,7 +1399,7 @@
         <v>5</v>
       </c>
       <c r="BN3" s="2">
-        <f t="shared" ref="BN3:BU3" si="6">ROUND(BZ8/BZ9,  1)</f>
+        <f t="shared" ref="BN3:BT3" si="6">ROUND(BZ8/BZ9,  1)</f>
         <v>5</v>
       </c>
       <c r="BO3" s="2">
@@ -1571,56 +1567,44 @@
       <c r="AC4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AD4" s="2">
-        <f t="shared" ref="AD4:AT4" si="8">ROUND(AP8/AP9,  1)</f>
-        <v>5</v>
-      </c>
-      <c r="AE4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AF4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AG4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AH4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AI4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AJ4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AK4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AL4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AM4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AN4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
-      </c>
-      <c r="AO4" s="2">
-        <f t="shared" si="8"/>
-        <v>5</v>
+      <c r="AD4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AE4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AF4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AH4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AI4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AJ4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AK4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AL4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AM4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AN4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AO4" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="AP4" s="2">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="AD4:AT4" si="8">ROUND(BB8/BB9,  1)</f>
         <v>5</v>
       </c>
       <c r="AQ4" s="2">
@@ -1640,7 +1624,7 @@
         <v>5</v>
       </c>
       <c r="AU4" s="2">
-        <f t="shared" ref="AU4:BU4" si="9">ROUND(BG8/BG9,  1)</f>
+        <f t="shared" ref="AU4:BT4" si="9">ROUND(BG8/BG9,  1)</f>
         <v>5</v>
       </c>
       <c r="AV4" s="2">
@@ -2673,7 +2657,7 @@
         <v>3</v>
       </c>
       <c r="B17" s="1">
-        <v>185.9</v>
+        <v>165.9</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -2681,7 +2665,7 @@
         <v>4</v>
       </c>
       <c r="B18" s="1">
-        <v>1</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>